<commit_message>
Option to specify subjects for ROI analysis. Single model specification removed from step 8 (localizer only).
</commit_message>
<xml_diff>
--- a/pipeline/second_level_roi/roi_coordinates.xlsx
+++ b/pipeline/second_level_roi/roi_coordinates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\thesis-matlab-pipeline\pipeline\second_level_roi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02A9DBFF-B1AA-46B1-9B6F-65310EF125EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65F8F63C-FF53-4256-8FE0-5666E35EB4FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="66">
   <si>
     <t>participant_id</t>
   </si>
@@ -62,21 +62,12 @@
     <t>JF</t>
   </si>
   <si>
-    <t>42 -52 -20</t>
-  </si>
-  <si>
     <t>42 -54 -18</t>
   </si>
   <si>
     <t>46 -56 -20</t>
   </si>
   <si>
-    <t>!: not detected in localizer</t>
-  </si>
-  <si>
-    <t>-42 -82 10</t>
-  </si>
-  <si>
     <t>44 -78 -4</t>
   </si>
   <si>
@@ -92,9 +83,6 @@
     <t>-38 -50 -20</t>
   </si>
   <si>
-    <t>42 -78 -6</t>
-  </si>
-  <si>
     <t>41 -72 -13</t>
   </si>
   <si>
@@ -104,18 +92,12 @@
     <t xml:space="preserve">40 -48 -22 </t>
   </si>
   <si>
-    <t>-42 -80 -10</t>
-  </si>
-  <si>
     <t>-40 -48 -22</t>
   </si>
   <si>
     <t>-41 -72 -13</t>
   </si>
   <si>
-    <t>-44 -68 -14</t>
-  </si>
-  <si>
     <t>34 -84 -8</t>
   </si>
   <si>
@@ -131,9 +113,6 @@
     <t>40 -80 -12</t>
   </si>
   <si>
-    <t>44 -60 -14</t>
-  </si>
-  <si>
     <t>-40 -52 -16</t>
   </si>
   <si>
@@ -143,24 +122,15 @@
     <t>-46 -58 -22</t>
   </si>
   <si>
-    <t>42 -44 -22</t>
-  </si>
-  <si>
     <t>38 -62 -12</t>
   </si>
   <si>
-    <t>-44 -80 -2</t>
-  </si>
-  <si>
     <t>52 -76 -4</t>
   </si>
   <si>
     <t>-40 -48 -22!</t>
   </si>
   <si>
-    <t>40 -48 -22!</t>
-  </si>
-  <si>
     <t>44 -74 -8</t>
   </si>
   <si>
@@ -188,15 +158,6 @@
     <t>48 -76 -2</t>
   </si>
   <si>
-    <t>-46 -80 -2</t>
-  </si>
-  <si>
-    <t>-44 -76 -16</t>
-  </si>
-  <si>
-    <t>40 -56 -14</t>
-  </si>
-  <si>
     <t>44 -82 -8</t>
   </si>
   <si>
@@ -216,6 +177,63 @@
   </si>
   <si>
     <t>left_OFA</t>
+  </si>
+  <si>
+    <t>42 -80 -10</t>
+  </si>
+  <si>
+    <t>-44 -52 -24</t>
+  </si>
+  <si>
+    <t>-44 -82 -10</t>
+  </si>
+  <si>
+    <t>-38 -76 -18</t>
+  </si>
+  <si>
+    <t>-44 -78 - 10</t>
+  </si>
+  <si>
+    <t>-40 -78 -20</t>
+  </si>
+  <si>
+    <t>-42 -84 -8</t>
+  </si>
+  <si>
+    <t>-40 -48 -24</t>
+  </si>
+  <si>
+    <t>36 -50 -16</t>
+  </si>
+  <si>
+    <t>-42 -54 -20</t>
+  </si>
+  <si>
+    <t>areas not found, default coordinates</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>+</t>
+  </si>
+  <si>
+    <t>44 -52 -20</t>
+  </si>
+  <si>
+    <t>44 -58 -14</t>
+  </si>
+  <si>
+    <t>44 -44 -22</t>
+  </si>
+  <si>
+    <t>38 -52 -18</t>
+  </si>
+  <si>
+    <t>38 -42 -16</t>
+  </si>
+  <si>
+    <t>40 -52 -22</t>
   </si>
 </sst>
 </file>
@@ -534,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -544,7 +562,7 @@
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -552,39 +570,45 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="E1" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="F1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -592,19 +616,22 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="G3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -612,19 +639,22 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="G4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -632,19 +662,22 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>13</v>
-      </c>
       <c r="F5" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="G5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -652,19 +685,22 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="G6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -672,19 +708,22 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="G7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -692,117 +731,127 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="G8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+      <c r="G9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="E11" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="G11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="E12" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+      <c r="G12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C15" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed ROI extraction script to overwrite existing ROI-spheres to enable more flexible analysis. Renamed ROI plot and statistics scripts for clarity.
</commit_message>
<xml_diff>
--- a/pipeline/second_level_roi/roi_coordinates.xlsx
+++ b/pipeline/second_level_roi/roi_coordinates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\thesis-matlab-pipeline\pipeline\second_level_roi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A20996-FFE3-4AD8-9B1E-0D64BBCA24E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DE246C0-E118-4754-AC4C-5B22633ACD6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7275" yWindow="2475" windowWidth="14490" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="107">
   <si>
     <t>participant_id</t>
   </si>
@@ -77,9 +77,6 @@
     <t>-38 -74 -4</t>
   </si>
   <si>
-    <t>50 -74 - 10</t>
-  </si>
-  <si>
     <t>-38 -50 -20</t>
   </si>
   <si>
@@ -116,15 +113,9 @@
     <t>-40 -52 -16</t>
   </si>
   <si>
-    <t>-46 -74 -14</t>
-  </si>
-  <si>
     <t>-46 -58 -22</t>
   </si>
   <si>
-    <t>38 -62 -12</t>
-  </si>
-  <si>
     <t>52 -76 -4</t>
   </si>
   <si>
@@ -185,39 +176,12 @@
     <t>-44 -52 -24</t>
   </si>
   <si>
-    <t>-44 -82 -10</t>
-  </si>
-  <si>
-    <t>-38 -76 -18</t>
-  </si>
-  <si>
-    <t>-44 -78 - 10</t>
-  </si>
-  <si>
-    <t>-40 -78 -20</t>
-  </si>
-  <si>
-    <t>-42 -84 -8</t>
-  </si>
-  <si>
-    <t>-40 -48 -24</t>
-  </si>
-  <si>
     <t>36 -50 -16</t>
   </si>
   <si>
     <t>-42 -54 -20</t>
   </si>
   <si>
-    <t>areas not found, default coordinates</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>+</t>
-  </si>
-  <si>
     <t>44 -52 -20</t>
   </si>
   <si>
@@ -242,9 +206,6 @@
     <t>-42 -82 -6</t>
   </si>
   <si>
-    <t>-38 -54 -18</t>
-  </si>
-  <si>
     <t>42 -82 -10</t>
   </si>
   <si>
@@ -260,9 +221,6 @@
     <t>-44 -58 -16</t>
   </si>
   <si>
-    <t>-52 -68 -8</t>
-  </si>
-  <si>
     <t>50 -72 -14</t>
   </si>
   <si>
@@ -275,9 +233,6 @@
     <t>46 -80 -8</t>
   </si>
   <si>
-    <t>-40 -82 -2</t>
-  </si>
-  <si>
     <t>-42 -54 -18</t>
   </si>
   <si>
@@ -288,16 +243,136 @@
   </si>
   <si>
     <t>42 -60 -18</t>
+  </si>
+  <si>
+    <t>KR</t>
+  </si>
+  <si>
+    <t>-38 -60 -18</t>
+  </si>
+  <si>
+    <t>-34 -90 -14</t>
+  </si>
+  <si>
+    <t>42 -62 -18</t>
+  </si>
+  <si>
+    <t>48 -78 -8</t>
+  </si>
+  <si>
+    <t>LM</t>
+  </si>
+  <si>
+    <t>-46 -78 -12</t>
+  </si>
+  <si>
+    <t>40 -50 -22</t>
+  </si>
+  <si>
+    <t>-40 -54 -20</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>vp01</t>
+  </si>
+  <si>
+    <t>vp02</t>
+  </si>
+  <si>
+    <t>vp03</t>
+  </si>
+  <si>
+    <t>vp04</t>
+  </si>
+  <si>
+    <t>vp05</t>
+  </si>
+  <si>
+    <t>vp06</t>
+  </si>
+  <si>
+    <t>vp07</t>
+  </si>
+  <si>
+    <t>vp08</t>
+  </si>
+  <si>
+    <t>vp09_MH</t>
+  </si>
+  <si>
+    <t>vp10_YM</t>
+  </si>
+  <si>
+    <t>vp11_KL</t>
+  </si>
+  <si>
+    <t>vp13_HG</t>
+  </si>
+  <si>
+    <t>vp12_AJ</t>
+  </si>
+  <si>
+    <t>vp14_UM</t>
+  </si>
+  <si>
+    <t>vp15_LJ</t>
+  </si>
+  <si>
+    <t>vp16_KR</t>
+  </si>
+  <si>
+    <t>vp17_LM</t>
+  </si>
+  <si>
+    <t>-48 -82 -10</t>
+  </si>
+  <si>
+    <t>-42 -76 -4</t>
+  </si>
+  <si>
+    <t>-44 -80 -2</t>
+  </si>
+  <si>
+    <t>-44 -56 -18</t>
+  </si>
+  <si>
+    <t>-46 -80 2</t>
+  </si>
+  <si>
+    <t>-36 -58 -16</t>
+  </si>
+  <si>
+    <t>-40 -86 -10</t>
+  </si>
+  <si>
+    <t>-38 -80 -14</t>
+  </si>
+  <si>
+    <t>44 -78 -12</t>
+  </si>
+  <si>
+    <t>50 -74 -10</t>
+  </si>
+  <si>
+    <t>-44 -78 -10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -606,7 +681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -614,9 +689,10 @@
     <col min="3" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -624,45 +700,45 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" t="s">
         <v>43</v>
       </c>
-      <c r="D1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -670,22 +746,22 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -693,22 +769,22 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D4" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -716,22 +792,22 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="E5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G5" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -739,22 +815,22 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -762,22 +838,22 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -785,194 +861,253 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>27</v>
+        <v>85</v>
+      </c>
+      <c r="D8" t="s">
+        <v>50</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E9" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+      <c r="D9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>65</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G11" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+      <c r="D11" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" t="s">
+        <v>37</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E12" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G12" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+      <c r="D12" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" t="s">
+        <v>28</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+      <c r="D13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>72</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="D14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>76</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E15" t="s">
-        <v>78</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+      <c r="D15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F15" t="s">
+        <v>64</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" t="s">
+        <v>68</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F16" t="s">
+        <v>66</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" t="s">
+        <v>72</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E16" t="s">
-        <v>81</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>82</v>
+      <c r="F17" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" t="s">
+        <v>104</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Added improved scripts for ROI second level statistics and plots. Added helper scripts for 5 condition analysis. Modified ROI analysis scripts.
</commit_message>
<xml_diff>
--- a/pipeline/second_level_roi/roi_coordinates.xlsx
+++ b/pipeline/second_level_roi/roi_coordinates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\thesis-matlab-pipeline\pipeline\second_level_roi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DE246C0-E118-4754-AC4C-5B22633ACD6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B1F71B-42E6-4F7C-8961-A7749D79299C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="113">
   <si>
     <t>participant_id</t>
   </si>
@@ -119,9 +119,6 @@
     <t>52 -76 -4</t>
   </si>
   <si>
-    <t>-40 -48 -22!</t>
-  </si>
-  <si>
     <t>44 -74 -8</t>
   </si>
   <si>
@@ -170,12 +167,6 @@
     <t>left_OFA</t>
   </si>
   <si>
-    <t>42 -80 -10</t>
-  </si>
-  <si>
-    <t>-44 -52 -24</t>
-  </si>
-  <si>
     <t>36 -50 -16</t>
   </si>
   <si>
@@ -233,9 +224,6 @@
     <t>46 -80 -8</t>
   </si>
   <si>
-    <t>-42 -54 -18</t>
-  </si>
-  <si>
     <t>44 -78 -6</t>
   </si>
   <si>
@@ -251,9 +239,6 @@
     <t>-38 -60 -18</t>
   </si>
   <si>
-    <t>-34 -90 -14</t>
-  </si>
-  <si>
     <t>42 -62 -18</t>
   </si>
   <si>
@@ -344,9 +329,6 @@
     <t>-36 -58 -16</t>
   </si>
   <si>
-    <t>-40 -86 -10</t>
-  </si>
-  <si>
     <t>-38 -80 -14</t>
   </si>
   <si>
@@ -357,6 +339,42 @@
   </si>
   <si>
     <t>-44 -78 -10</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>vp18_LS</t>
+  </si>
+  <si>
+    <t>-42 -46 -22</t>
+  </si>
+  <si>
+    <t>40 -54 -18</t>
+  </si>
+  <si>
+    <t>46 -76 4</t>
+  </si>
+  <si>
+    <t>-44 -54 -22</t>
+  </si>
+  <si>
+    <t>42 -80 -12</t>
+  </si>
+  <si>
+    <t>-40 -48 -24</t>
+  </si>
+  <si>
+    <t>-42 -82 2</t>
+  </si>
+  <si>
+    <t>-40 -44 -26</t>
+  </si>
+  <si>
+    <t>-36 -90 -14</t>
+  </si>
+  <si>
+    <t>-50 -76 -6</t>
   </si>
 </sst>
 </file>
@@ -378,12 +396,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -398,9 +428,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -681,7 +714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -700,19 +733,19 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" t="s">
         <v>40</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>41</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>42</v>
-      </c>
-      <c r="G1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -723,7 +756,7 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D2" t="s">
         <v>16</v>
@@ -734,7 +767,7 @@
       <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="4" t="s">
         <v>18</v>
       </c>
     </row>
@@ -746,19 +779,19 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>96</v>
+      <c r="E3" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -769,16 +802,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>12</v>
@@ -792,7 +825,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D5" t="s">
         <v>9</v>
@@ -804,7 +837,7 @@
         <v>10</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -815,7 +848,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
         <v>20</v>
@@ -838,10 +871,10 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>24</v>
@@ -850,7 +883,7 @@
         <v>23</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -861,19 +894,19 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>25</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -881,22 +914,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F9" t="s">
         <v>35</v>
       </c>
-      <c r="C9" t="s">
-        <v>86</v>
-      </c>
-      <c r="D9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F9" t="s">
-        <v>36</v>
-      </c>
       <c r="G9" s="1" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -904,16 +937,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>27</v>
+        <v>49</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>108</v>
       </c>
       <c r="F10" t="s">
         <v>26</v>
@@ -927,22 +960,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -950,22 +983,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F12" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,22 +1006,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D13" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F13" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -996,22 +1029,22 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>57</v>
       </c>
       <c r="F14" t="s">
-        <v>61</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>102</v>
+        <v>58</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1019,22 +1052,22 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>60</v>
       </c>
       <c r="F15" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1042,22 +1075,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C16" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="F16" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1065,22 +1098,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C17" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D17" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F17" t="s">
-        <v>73</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1088,22 +1121,45 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F18" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" t="s">
         <v>104</v>
       </c>
-      <c r="G18" s="1" t="s">
-        <v>75</v>
+      <c r="E19" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F19" t="s">
+        <v>105</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>